<commit_message>
Revise homework 1 report after data and language review
Remove the reference list, citation marks and code appendix; correct
the Q-Q, PCA and cluster interpretations flagged by an independent
recomputation; use half-up rounding, a consistent minus sign and
italic statistical symbols; tighten the prose.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012tanStY1L9RUWAxoKiPCX6
</commit_message>
<xml_diff>
--- a/作业一_五个班级成绩数据挖掘/成绩数据_清洗后及分析结果.xlsx
+++ b/作业一_五个班级成绩数据挖掘/成绩数据_清洗后及分析结果.xlsx
@@ -62,7 +62,7 @@
     <t>课程平均分</t>
   </si>
   <si>
-    <t>是否挂科</t>
+    <t>是否不及格</t>
   </si>
   <si>
     <t>成绩等级</t>
@@ -659,7 +659,7 @@
     <t>A 学业优良组</t>
   </si>
   <si>
-    <t>B 稳定中等组</t>
+    <t>B 中等组</t>
   </si>
   <si>
     <t>C 学业预警组</t>
@@ -713,7 +713,7 @@
     <t>百分号文本(如 82.14%)</t>
   </si>
   <si>
-    <t>小数文本(如 0.8)</t>
+    <t>数值型小数(单元格显示为百分比)</t>
   </si>
   <si>
     <t>均值</t>
@@ -779,10 +779,10 @@
     <t>课程平均分(均值)</t>
   </si>
   <si>
-    <t>挂科人数</t>
-  </si>
-  <si>
-    <t>挂科率</t>
+    <t>不及格人数</t>
+  </si>
+  <si>
+    <t>不及格率</t>
   </si>
   <si>
     <t>不及格门次合计</t>

</xml_diff>

<commit_message>
Final review pass on homework 1 report
Resolve the four final reviews: redraw figures at print size with
consistent fonts, minus signs, colour meanings and half-up labels;
redraw the parallel-coordinates plot per student as described in
class; drop the PCA projection; remove duplicated and defensive
sentences; correct the pass-rate, Q-Q and k = 4 interpretations;
place cluster evaluation before the warning list.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012tanStY1L9RUWAxoKiPCX6
</commit_message>
<xml_diff>
--- a/作业一_五个班级成绩数据挖掘/成绩数据_清洗后及分析结果.xlsx
+++ b/作业一_五个班级成绩数据挖掘/成绩数据_清洗后及分析结果.xlsx
@@ -12,19 +12,18 @@
     <sheet name="描述统计_加权平均分" sheetId="3" r:id="rId3"/>
     <sheet name="其他指标" sheetId="4" r:id="rId4"/>
     <sheet name="成绩等级人数" sheetId="5" r:id="rId5"/>
-    <sheet name="两两比较" sheetId="6" r:id="rId6"/>
-    <sheet name="异常点" sheetId="7" r:id="rId7"/>
-    <sheet name="相关系数" sheetId="8" r:id="rId8"/>
-    <sheet name="聚类画像" sheetId="9" r:id="rId9"/>
-    <sheet name="聚类×班级" sheetId="10" r:id="rId10"/>
-    <sheet name="学业预警名单" sheetId="11" r:id="rId11"/>
+    <sheet name="异常点" sheetId="6" r:id="rId6"/>
+    <sheet name="相关系数" sheetId="7" r:id="rId7"/>
+    <sheet name="聚类画像" sheetId="8" r:id="rId8"/>
+    <sheet name="聚类×班级" sheetId="9" r:id="rId9"/>
+    <sheet name="学业预警名单" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="958" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="922" uniqueCount="257">
   <si>
     <t>班级</t>
   </si>
@@ -792,30 +791,6 @@
   </si>
   <si>
     <t>通过率(均值)</t>
-  </si>
-  <si>
-    <t>班级A</t>
-  </si>
-  <si>
-    <t>班级B</t>
-  </si>
-  <si>
-    <t>中位数差(A-B)</t>
-  </si>
-  <si>
-    <t>p值</t>
-  </si>
-  <si>
-    <t>Holm校正p值</t>
-  </si>
-  <si>
-    <t>显著(α=0.05)</t>
-  </si>
-  <si>
-    <t>是</t>
-  </si>
-  <si>
-    <t>否</t>
   </si>
   <si>
     <t>人数</t>
@@ -13869,100 +13844,6 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>210</v>
-      </c>
-      <c r="C1" t="s">
-        <v>211</v>
-      </c>
-      <c r="D1" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2">
-        <v>5</v>
-      </c>
-      <c r="C2">
-        <v>18</v>
-      </c>
-      <c r="D2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3">
-        <v>7</v>
-      </c>
-      <c r="C3">
-        <v>22</v>
-      </c>
-      <c r="D3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4">
-        <v>27</v>
-      </c>
-      <c r="C4">
-        <v>3</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5">
-        <v>17</v>
-      </c>
-      <c r="C5">
-        <v>22</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6">
-        <v>17</v>
-      </c>
-      <c r="C6">
-        <v>18</v>
-      </c>
-      <c r="D6">
-        <v>4</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -15415,227 +15296,137 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
-        <v>256</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>257</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>258</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>259</v>
+        <v>6</v>
       </c>
       <c r="E1" t="s">
-        <v>260</v>
+        <v>5</v>
       </c>
       <c r="F1" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="C2">
-        <v>-10.74499999999999</v>
+        <v>61.93</v>
       </c>
       <c r="D2">
-        <v>1.532744598360007E-10</v>
+        <v>1.43</v>
       </c>
       <c r="E2">
-        <v>1.532744598360007E-09</v>
-      </c>
-      <c r="F2" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>11</v>
+      </c>
+      <c r="G2">
+        <v>0.6071</v>
+      </c>
+      <c r="H2">
+        <v>-2.929244840835825</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="C3">
-        <v>-9.279999999999987</v>
+        <v>65.06999999999999</v>
       </c>
       <c r="D3">
-        <v>2.101528092640487E-08</v>
+        <v>1.68</v>
       </c>
       <c r="E3">
-        <v>1.891375283376438E-07</v>
-      </c>
-      <c r="F3" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>3</v>
+      </c>
+      <c r="F3">
+        <v>13</v>
+      </c>
+      <c r="G3">
+        <v>0.5357</v>
+      </c>
+      <c r="H3">
+        <v>-2.53991480842651</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C4">
+        <v>67.68000000000001</v>
+      </c>
+      <c r="D4">
+        <v>1.76</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>10</v>
+      </c>
+      <c r="G4">
+        <v>0.6</v>
+      </c>
+      <c r="H4">
+        <v>-2.672228053404945</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
         <v>27</v>
       </c>
-      <c r="C4">
-        <v>5.965000000000003</v>
-      </c>
-      <c r="D4">
-        <v>7.422965184183506E-08</v>
-      </c>
-      <c r="E4">
-        <v>5.938372147346805E-07</v>
-      </c>
-      <c r="F4" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>25</v>
-      </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>205</v>
       </c>
       <c r="C5">
-        <v>6.265000000000001</v>
+        <v>68.84</v>
       </c>
       <c r="D5">
-        <v>4.285396582531695E-07</v>
+        <v>1.62</v>
       </c>
       <c r="E5">
-        <v>2.999777607772186E-06</v>
-      </c>
-      <c r="F5" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6">
-        <v>-4.47999999999999</v>
-      </c>
-      <c r="D6">
-        <v>9.505052606917286E-05</v>
-      </c>
-      <c r="E6">
-        <v>0.0005703031564150371</v>
-      </c>
-      <c r="F6" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7">
-        <v>-4.779999999999987</v>
-      </c>
-      <c r="D7">
-        <v>0.0008212529182532857</v>
-      </c>
-      <c r="E7">
-        <v>0.004106264591266428</v>
-      </c>
-      <c r="F7" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8">
-        <v>-3.014999999999986</v>
-      </c>
-      <c r="D8">
-        <v>0.008262564563951693</v>
-      </c>
-      <c r="E8">
-        <v>0.03305025825580677</v>
-      </c>
-      <c r="F8" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9">
-        <v>-3.314999999999984</v>
-      </c>
-      <c r="D9">
-        <v>0.04775431803205206</v>
-      </c>
-      <c r="E9">
-        <v>0.1432629540961562</v>
-      </c>
-      <c r="F9" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10">
-        <v>-1.465000000000003</v>
-      </c>
-      <c r="D10">
-        <v>0.2668771321503037</v>
-      </c>
-      <c r="E10">
-        <v>0.5337542643006075</v>
-      </c>
-      <c r="F10" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11">
-        <v>-0.2999999999999972</v>
-      </c>
-      <c r="D11">
-        <v>0.6696957769319646</v>
-      </c>
-      <c r="E11">
-        <v>0.6696957769319646</v>
-      </c>
-      <c r="F11" t="s">
-        <v>263</v>
+        <v>3</v>
+      </c>
+      <c r="F5">
+        <v>11</v>
+      </c>
+      <c r="G5">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="H5">
+        <v>-2.442203703880554</v>
       </c>
     </row>
   </sheetData>
@@ -15645,137 +15436,265 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
+    <row r="1" spans="1:9">
       <c r="B1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>0.9926913370907693</v>
+      </c>
+      <c r="D2">
+        <v>0.9668115452511287</v>
+      </c>
+      <c r="E2">
+        <v>0.6562251029843983</v>
+      </c>
+      <c r="F2">
+        <v>0.5116800283340888</v>
+      </c>
+      <c r="G2">
+        <v>-0.6417131870354394</v>
+      </c>
+      <c r="H2">
+        <v>-0.6420700802208283</v>
+      </c>
+      <c r="I2">
+        <v>0.6402242531077101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="E1" t="s">
+      <c r="B3">
+        <v>0.9926913370907693</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>0.9607244332348207</v>
+      </c>
+      <c r="E3">
+        <v>0.6622534947933415</v>
+      </c>
+      <c r="F3">
+        <v>0.4889094178375819</v>
+      </c>
+      <c r="G3">
+        <v>-0.6123670629362454</v>
+      </c>
+      <c r="H3">
+        <v>-0.611158205247217</v>
+      </c>
+      <c r="I3">
+        <v>0.612797902541245</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4">
+        <v>0.9668115452511287</v>
+      </c>
+      <c r="C4">
+        <v>0.9607244332348207</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>0.6865724332021343</v>
+      </c>
+      <c r="F4">
+        <v>0.5075085761728477</v>
+      </c>
+      <c r="G4">
+        <v>-0.6203278342607325</v>
+      </c>
+      <c r="H4">
+        <v>-0.6460062306538887</v>
+      </c>
+      <c r="I4">
+        <v>0.6204933590913775</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <v>0.6562251029843983</v>
+      </c>
+      <c r="C5">
+        <v>0.6622534947933415</v>
+      </c>
+      <c r="D5">
+        <v>0.6865724332021343</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>0.6551462547475</v>
+      </c>
+      <c r="G5">
+        <v>-0.3513413294956685</v>
+      </c>
+      <c r="H5">
+        <v>-0.3675403930021223</v>
+      </c>
+      <c r="I5">
+        <v>0.3629009604737863</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6">
+        <v>0.5116800283340888</v>
+      </c>
+      <c r="C6">
+        <v>0.4889094178375819</v>
+      </c>
+      <c r="D6">
+        <v>0.5075085761728477</v>
+      </c>
+      <c r="E6">
+        <v>0.6551462547475</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>-0.8419214868918019</v>
+      </c>
+      <c r="H6">
+        <v>-0.8084278427755311</v>
+      </c>
+      <c r="I6">
+        <v>0.8504232680973955</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7">
+        <v>-0.6417131870354394</v>
+      </c>
+      <c r="C7">
+        <v>-0.6123670629362454</v>
+      </c>
+      <c r="D7">
+        <v>-0.6203278342607325</v>
+      </c>
+      <c r="E7">
+        <v>-0.3513413294956685</v>
+      </c>
+      <c r="F7">
+        <v>-0.8419214868918019</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>0.9653323664584884</v>
+      </c>
+      <c r="I7">
+        <v>-0.9984235542771239</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
         <v>5</v>
       </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="B8">
+        <v>-0.6420700802208283</v>
+      </c>
+      <c r="C8">
+        <v>-0.611158205247217</v>
+      </c>
+      <c r="D8">
+        <v>-0.6460062306538887</v>
+      </c>
+      <c r="E8">
+        <v>-0.3675403930021223</v>
+      </c>
+      <c r="F8">
+        <v>-0.8084278427755311</v>
+      </c>
+      <c r="G8">
+        <v>0.9653323664584884</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>-0.9640850569561594</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="H1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C2">
-        <v>61.93</v>
-      </c>
-      <c r="D2">
-        <v>1.43</v>
-      </c>
-      <c r="E2">
-        <v>4</v>
-      </c>
-      <c r="F2">
-        <v>11</v>
-      </c>
-      <c r="G2">
-        <v>0.6071</v>
-      </c>
-      <c r="H2">
-        <v>-2.929244840835825</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" t="s">
-        <v>96</v>
-      </c>
-      <c r="C3">
-        <v>65.06999999999999</v>
-      </c>
-      <c r="D3">
-        <v>1.68</v>
-      </c>
-      <c r="E3">
-        <v>3</v>
-      </c>
-      <c r="F3">
-        <v>13</v>
-      </c>
-      <c r="G3">
-        <v>0.5357</v>
-      </c>
-      <c r="H3">
-        <v>-2.53991480842651</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" t="s">
-        <v>204</v>
-      </c>
-      <c r="C4">
-        <v>67.68000000000001</v>
-      </c>
-      <c r="D4">
-        <v>1.76</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="F4">
-        <v>10</v>
-      </c>
-      <c r="G4">
-        <v>0.6</v>
-      </c>
-      <c r="H4">
-        <v>-2.672228053404945</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" t="s">
-        <v>205</v>
-      </c>
-      <c r="C5">
-        <v>68.84</v>
-      </c>
-      <c r="D5">
-        <v>1.62</v>
-      </c>
-      <c r="E5">
-        <v>3</v>
-      </c>
-      <c r="F5">
-        <v>11</v>
-      </c>
-      <c r="G5">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="H5">
-        <v>-2.442203703880554</v>
+      <c r="B9">
+        <v>0.6402242531077101</v>
+      </c>
+      <c r="C9">
+        <v>0.612797902541245</v>
+      </c>
+      <c r="D9">
+        <v>0.6204933590913775</v>
+      </c>
+      <c r="E9">
+        <v>0.3629009604737863</v>
+      </c>
+      <c r="F9">
+        <v>0.8504232680973955</v>
+      </c>
+      <c r="G9">
+        <v>-0.9984235542771239</v>
+      </c>
+      <c r="H9">
+        <v>-0.9640850569561594</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -15785,265 +15704,99 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>22</v>
+      </c>
       <c r="B1" t="s">
+        <v>256</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" t="s">
-        <v>11</v>
-      </c>
       <c r="E1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>210</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>73</v>
       </c>
       <c r="C2">
-        <v>0.9926913370907693</v>
+        <v>86.6804109589041</v>
       </c>
       <c r="D2">
-        <v>0.9668115452511287</v>
+        <v>3.495205479452055</v>
       </c>
       <c r="E2">
-        <v>0.6562251029843983</v>
+        <v>0</v>
       </c>
       <c r="F2">
-        <v>0.5116800283340888</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>-0.6417131870354394</v>
-      </c>
-      <c r="H2">
-        <v>-0.6420700802208283</v>
-      </c>
-      <c r="I2">
-        <v>0.6402242531077101</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="B3">
-        <v>0.9926913370907693</v>
+        <v>83</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>78.93975903614458</v>
       </c>
       <c r="D3">
-        <v>0.9607244332348207</v>
+        <v>2.723493975903615</v>
       </c>
       <c r="E3">
-        <v>0.6622534947933415</v>
+        <v>0.02409638554216868</v>
       </c>
       <c r="F3">
-        <v>0.4889094178375819</v>
+        <v>0.04819277108433735</v>
       </c>
       <c r="G3">
-        <v>-0.6123670629362454</v>
-      </c>
-      <c r="H3">
-        <v>-0.611158205247217</v>
-      </c>
-      <c r="I3">
-        <v>0.612797902541245</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
+        <v>0.9982795180722892</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>212</v>
       </c>
       <c r="B4">
-        <v>0.9668115452511287</v>
+        <v>22</v>
       </c>
       <c r="C4">
-        <v>0.9607244332348207</v>
+        <v>71.64636363636363</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>2.048636363636364</v>
       </c>
       <c r="E4">
-        <v>0.6865724332021343</v>
+        <v>1.636363636363636</v>
       </c>
       <c r="F4">
-        <v>0.5075085761728477</v>
+        <v>6.954545454545454</v>
       </c>
       <c r="G4">
-        <v>-0.6203278342607325</v>
-      </c>
-      <c r="H4">
-        <v>-0.6460062306538887</v>
-      </c>
-      <c r="I4">
-        <v>0.6204933590913775</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5">
-        <v>0.6562251029843983</v>
-      </c>
-      <c r="C5">
-        <v>0.6622534947933415</v>
-      </c>
-      <c r="D5">
-        <v>0.6865724332021343</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>0.6551462547475</v>
-      </c>
-      <c r="G5">
-        <v>-0.3513413294956685</v>
-      </c>
-      <c r="H5">
-        <v>-0.3675403930021223</v>
-      </c>
-      <c r="I5">
-        <v>0.3629009604737863</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6">
-        <v>0.5116800283340888</v>
-      </c>
-      <c r="C6">
-        <v>0.4889094178375819</v>
-      </c>
-      <c r="D6">
-        <v>0.5075085761728477</v>
-      </c>
-      <c r="E6">
-        <v>0.6551462547475</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6">
-        <v>-0.8419214868918019</v>
-      </c>
-      <c r="H6">
-        <v>-0.8084278427755311</v>
-      </c>
-      <c r="I6">
-        <v>0.8504232680973955</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7">
-        <v>-0.6417131870354394</v>
-      </c>
-      <c r="C7">
-        <v>-0.6123670629362454</v>
-      </c>
-      <c r="D7">
-        <v>-0.6203278342607325</v>
-      </c>
-      <c r="E7">
-        <v>-0.3513413294956685</v>
-      </c>
-      <c r="F7">
-        <v>-0.8419214868918019</v>
-      </c>
-      <c r="G7">
-        <v>1</v>
-      </c>
-      <c r="H7">
-        <v>0.9653323664584884</v>
-      </c>
-      <c r="I7">
-        <v>-0.9984235542771239</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="A8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8">
-        <v>-0.6420700802208283</v>
-      </c>
-      <c r="C8">
-        <v>-0.611158205247217</v>
-      </c>
-      <c r="D8">
-        <v>-0.6460062306538887</v>
-      </c>
-      <c r="E8">
-        <v>-0.3675403930021223</v>
-      </c>
-      <c r="F8">
-        <v>-0.8084278427755311</v>
-      </c>
-      <c r="G8">
-        <v>0.9653323664584884</v>
-      </c>
-      <c r="H8">
-        <v>1</v>
-      </c>
-      <c r="I8">
-        <v>-0.9640850569561594</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>0.6402242531077101</v>
-      </c>
-      <c r="C9">
-        <v>0.612797902541245</v>
-      </c>
-      <c r="D9">
-        <v>0.6204933590913775</v>
-      </c>
-      <c r="E9">
-        <v>0.3629009604737863</v>
-      </c>
-      <c r="F9">
-        <v>0.8504232680973955</v>
-      </c>
-      <c r="G9">
-        <v>-0.9984235542771239</v>
-      </c>
-      <c r="H9">
-        <v>-0.9640850569561594</v>
-      </c>
-      <c r="I9">
-        <v>1</v>
+        <v>0.7430636363636364</v>
       </c>
     </row>
   </sheetData>
@@ -16053,99 +15806,91 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>210</v>
+      </c>
+      <c r="C1" t="s">
+        <v>211</v>
+      </c>
+      <c r="D1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>18</v>
+      </c>
+      <c r="D2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3">
+        <v>7</v>
+      </c>
+      <c r="C3">
         <v>22</v>
       </c>
-      <c r="B1" t="s">
-        <v>264</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="D3">
         <v>5</v>
       </c>
-      <c r="F1" t="s">
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4">
+        <v>27</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5">
+        <v>17</v>
+      </c>
+      <c r="C5">
+        <v>22</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6">
+        <v>17</v>
+      </c>
+      <c r="C6">
+        <v>18</v>
+      </c>
+      <c r="D6">
         <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>210</v>
-      </c>
-      <c r="B2">
-        <v>73</v>
-      </c>
-      <c r="C2">
-        <v>86.6804109589041</v>
-      </c>
-      <c r="D2">
-        <v>3.495205479452055</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>211</v>
-      </c>
-      <c r="B3">
-        <v>83</v>
-      </c>
-      <c r="C3">
-        <v>78.93975903614458</v>
-      </c>
-      <c r="D3">
-        <v>2.723493975903615</v>
-      </c>
-      <c r="E3">
-        <v>0.02409638554216868</v>
-      </c>
-      <c r="F3">
-        <v>0.04819277108433735</v>
-      </c>
-      <c r="G3">
-        <v>0.9982795180722892</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
-        <v>212</v>
-      </c>
-      <c r="B4">
-        <v>22</v>
-      </c>
-      <c r="C4">
-        <v>71.64636363636363</v>
-      </c>
-      <c r="D4">
-        <v>2.048636363636364</v>
-      </c>
-      <c r="E4">
-        <v>1.636363636363636</v>
-      </c>
-      <c r="F4">
-        <v>6.954545454545454</v>
-      </c>
-      <c r="G4">
-        <v>0.7430636363636364</v>
       </c>
     </row>
   </sheetData>

</xml_diff>